<commit_message>
Update: Sentence changes and edits to test cases
</commit_message>
<xml_diff>
--- a/IT23362680_Test cases.xlsx
+++ b/IT23362680_Test cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT23362680\test_automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ADE0F63-D075-476D-ACEA-886D4052028B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FD6A942-00D4-4AAB-8F10-54F94C8D889E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="408" yWindow="636" windowWidth="14484" windowHeight="11208" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GitHub" sheetId="1" r:id="rId1"/>
@@ -152,9 +152,6 @@
     <t>නෑ bro, මට බැහැ.</t>
   </si>
   <si>
-    <t>පොඩ්ඩක් හිටපන්, මම ඒක check කරලා කියන්නම්.</t>
-  </si>
-  <si>
     <t>Neg_0010</t>
   </si>
   <si>
@@ -888,6 +885,9 @@
   </si>
   <si>
     <t>Evidence: '9:00AM' is a time format; 'Rs. 500' and 'Rs. 1500k' are currency; 'BTW' is an acronym; 'Kasun' is a person name;</t>
+  </si>
+  <si>
+    <t>නාහ් bro, මට බහ.</t>
   </si>
 </sst>
 </file>
@@ -1330,12 +1330,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -1377,10 +1377,10 @@
         <v>5</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -1403,10 +1403,10 @@
         <v>11</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -1429,10 +1429,10 @@
         <v>11</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -1455,10 +1455,10 @@
         <v>11</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -1481,10 +1481,10 @@
         <v>11</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -1507,10 +1507,10 @@
         <v>11</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -1533,10 +1533,10 @@
         <v>11</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -1559,10 +1559,10 @@
         <v>11</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -1576,7 +1576,7 @@
         <v>38</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>39</v>
@@ -1585,10 +1585,10 @@
         <v>11</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -1605,1082 +1605,1082 @@
         <v>42</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>43</v>
+        <v>288</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="E11" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>47</v>
-      </c>
       <c r="F11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="5" t="s">
+      <c r="D12" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="E12" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E12" s="5" t="s">
-        <v>51</v>
-      </c>
       <c r="F12" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>55</v>
-      </c>
       <c r="F13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E14" s="5" t="s">
-        <v>59</v>
-      </c>
       <c r="F14" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C15" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="E15" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E15" s="4" t="s">
-        <v>63</v>
-      </c>
       <c r="F15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C16" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="E16" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E16" s="5" t="s">
-        <v>67</v>
-      </c>
       <c r="F16" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C17" s="4" t="s">
+      <c r="D17" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="E17" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="E17" s="4" t="s">
-        <v>71</v>
-      </c>
       <c r="F17" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="E18" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="E18" s="5" t="s">
-        <v>75</v>
-      </c>
       <c r="F18" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C19" s="4" t="s">
+      <c r="D19" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="E19" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E19" s="4" t="s">
-        <v>79</v>
-      </c>
       <c r="F19" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="E20" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="E20" s="5" t="s">
-        <v>83</v>
-      </c>
       <c r="F20" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C21" s="4" t="s">
+      <c r="D21" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="E21" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="E21" s="4" t="s">
-        <v>87</v>
-      </c>
       <c r="F21" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="E22" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="E22" s="5" t="s">
-        <v>91</v>
-      </c>
       <c r="F22" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B23" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23" s="4" t="s">
+      <c r="D23" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="E23" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="E23" s="4" t="s">
-        <v>95</v>
-      </c>
       <c r="F23" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C24" s="5" t="s">
+      <c r="D24" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="E24" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="E24" s="5" t="s">
-        <v>99</v>
-      </c>
       <c r="F24" s="5" t="s">
         <v>11</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B25" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>101</v>
-      </c>
       <c r="D25" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C26" s="5" t="s">
+      <c r="D26" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="E26" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="E26" s="5" t="s">
-        <v>105</v>
-      </c>
       <c r="F26" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B27" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C27" s="4" t="s">
+      <c r="D27" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="E27" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E27" s="4" t="s">
-        <v>109</v>
-      </c>
       <c r="F27" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C28" s="5" t="s">
+      <c r="D28" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="E28" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="E28" s="5" t="s">
-        <v>113</v>
-      </c>
       <c r="F28" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="B29" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C29" s="4" t="s">
+      <c r="D29" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="E29" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="E29" s="4" t="s">
-        <v>117</v>
-      </c>
       <c r="F29" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C30" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="E30" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="E30" s="5" t="s">
-        <v>121</v>
-      </c>
       <c r="F30" s="5" t="s">
         <v>11</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B31" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C31" s="4" t="s">
+      <c r="D31" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="E31" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="E31" s="4" t="s">
-        <v>125</v>
-      </c>
       <c r="F31" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C32" s="5" t="s">
+      <c r="D32" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="E32" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="E32" s="5" t="s">
-        <v>129</v>
-      </c>
       <c r="F32" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C33" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="B33" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C33" s="4" t="s">
+      <c r="D33" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="E33" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="E33" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="F33" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C34" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C34" s="5" t="s">
+      <c r="D34" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="E34" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="E34" s="5" t="s">
-        <v>137</v>
-      </c>
       <c r="F34" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C35" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="B35" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C35" s="4" t="s">
+      <c r="D35" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="D35" s="4" t="s">
+      <c r="E35" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="E35" s="4" t="s">
-        <v>141</v>
-      </c>
       <c r="F35" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C36" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="E36" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="D36" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>206</v>
-      </c>
       <c r="F36" s="5" t="s">
         <v>11</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="B37" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C37" s="4" t="s">
+      <c r="D37" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="D37" s="4" t="s">
+      <c r="E37" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="E37" s="4" t="s">
-        <v>146</v>
-      </c>
       <c r="F37" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C38" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C38" s="5" t="s">
+      <c r="D38" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="E38" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="E38" s="5" t="s">
-        <v>150</v>
-      </c>
       <c r="F38" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C39" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="B39" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C39" s="4" t="s">
+      <c r="D39" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="D39" s="4" t="s">
+      <c r="E39" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="E39" s="4" t="s">
-        <v>154</v>
-      </c>
       <c r="F39" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C40" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="B40" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C40" s="5" t="s">
+      <c r="D40" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="E40" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="E40" s="5" t="s">
-        <v>158</v>
-      </c>
       <c r="F40" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C41" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="D41" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="D41" s="4" t="s">
+      <c r="E41" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="E41" s="4" t="s">
-        <v>162</v>
-      </c>
       <c r="F41" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C42" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C42" s="5" t="s">
+      <c r="D42" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="D42" s="5" t="s">
+      <c r="E42" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="E42" s="5" t="s">
-        <v>166</v>
-      </c>
       <c r="F42" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C43" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="B43" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C43" s="4" t="s">
+      <c r="D43" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="D43" s="4" t="s">
+      <c r="E43" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="E43" s="4" t="s">
-        <v>170</v>
-      </c>
       <c r="F43" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C44" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="B44" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C44" s="5" t="s">
+      <c r="D44" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="D44" s="5" t="s">
+      <c r="E44" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="E44" s="5" t="s">
-        <v>174</v>
-      </c>
       <c r="F44" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C45" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="B45" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C45" s="4" t="s">
+      <c r="D45" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="D45" s="4" t="s">
+      <c r="E45" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="E45" s="4" t="s">
-        <v>178</v>
-      </c>
       <c r="F45" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C46" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C46" s="5" t="s">
+      <c r="D46" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="D46" s="5" t="s">
-        <v>181</v>
-      </c>
       <c r="E46" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F46" s="5" t="s">
         <v>11</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C47" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="B47" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C47" s="4" t="s">
+      <c r="D47" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="D47" s="4" t="s">
-        <v>184</v>
-      </c>
       <c r="E47" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C48" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="B48" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C48" s="5" t="s">
+      <c r="D48" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="D48" s="5" t="s">
-        <v>188</v>
-      </c>
       <c r="E48" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C49" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="B49" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C49" s="4" t="s">
+      <c r="D49" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="D49" s="4" t="s">
-        <v>192</v>
-      </c>
       <c r="E49" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F49" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C50" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="B50" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C50" s="5" t="s">
+      <c r="D50" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="D50" s="5" t="s">
-        <v>196</v>
-      </c>
       <c r="E50" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F50" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G50" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H50" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="88.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="B51" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="B51" s="3" t="s">
+      <c r="C51" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="C51" s="4" t="s">
-        <v>199</v>
-      </c>
       <c r="D51" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F51" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
   </sheetData>

</xml_diff>